<commit_message>
updated working cells excel sheet and updated pick and place tasks that filters through the excel sheet to only have working cells
</commit_message>
<xml_diff>
--- a/fr3_real/fr3_100_cell_tracker.xlsx
+++ b/fr3_real/fr3_100_cell_tracker.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="14">
   <si>
     <t xml:space="preserve">printed_cell</t>
   </si>
@@ -56,6 +56,12 @@
   </si>
   <si>
     <t xml:space="preserve">grasp_tcp_z_m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PASS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FAIL</t>
   </si>
 </sst>
 </file>
@@ -172,7 +178,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -180,7 +186,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -339,7 +345,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="n">
         <v>1</v>
       </c>
@@ -355,7 +361,9 @@
       <c r="E2" s="0" t="n">
         <v>0</v>
       </c>
-      <c r="F2" s="2"/>
+      <c r="F2" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H2" s="0" t="n">
         <v>0.2608</v>
       </c>
@@ -372,7 +380,7 @@
         <v>0.0471</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="n">
         <v>2</v>
       </c>
@@ -388,7 +396,9 @@
       <c r="E3" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="F3" s="2"/>
+      <c r="F3" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H3" s="0" t="n">
         <v>0.2566</v>
       </c>
@@ -405,7 +415,7 @@
         <v>0.0459</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="n">
         <v>3</v>
       </c>
@@ -421,7 +431,9 @@
       <c r="E4" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="F4" s="2"/>
+      <c r="F4" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H4" s="0" t="n">
         <v>0.2523</v>
       </c>
@@ -438,7 +450,7 @@
         <v>0.0446</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="n">
         <v>4</v>
       </c>
@@ -454,7 +466,9 @@
       <c r="E5" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="F5" s="2"/>
+      <c r="F5" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H5" s="0" t="n">
         <v>0.248</v>
       </c>
@@ -471,7 +485,7 @@
         <v>0.0433</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="n">
         <v>5</v>
       </c>
@@ -487,7 +501,9 @@
       <c r="E6" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="F6" s="3"/>
+      <c r="F6" s="3" t="s">
+        <v>13</v>
+      </c>
       <c r="H6" s="0" t="n">
         <v>0.2438</v>
       </c>
@@ -504,7 +520,7 @@
         <v>0.042</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="n">
         <v>6</v>
       </c>
@@ -520,7 +536,9 @@
       <c r="E7" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="F7" s="4"/>
+      <c r="F7" s="3" t="s">
+        <v>13</v>
+      </c>
       <c r="H7" s="0" t="n">
         <v>0.2395</v>
       </c>
@@ -537,7 +555,7 @@
         <v>0.0407</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="n">
         <v>7</v>
       </c>
@@ -553,7 +571,9 @@
       <c r="E8" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="F8" s="4"/>
+      <c r="F8" s="3" t="s">
+        <v>13</v>
+      </c>
       <c r="H8" s="0" t="n">
         <v>0.2353</v>
       </c>
@@ -570,7 +590,7 @@
         <v>0.0394</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="n">
         <v>8</v>
       </c>
@@ -586,7 +606,9 @@
       <c r="E9" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="F9" s="4"/>
+      <c r="F9" s="3" t="s">
+        <v>13</v>
+      </c>
       <c r="H9" s="0" t="n">
         <v>0.231</v>
       </c>
@@ -603,7 +625,7 @@
         <v>0.0381</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="n">
         <v>9</v>
       </c>
@@ -619,7 +641,9 @@
       <c r="E10" s="0" t="n">
         <v>8</v>
       </c>
-      <c r="F10" s="2"/>
+      <c r="F10" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H10" s="0" t="n">
         <v>0.2267</v>
       </c>
@@ -636,7 +660,7 @@
         <v>0.0368</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="n">
         <v>10</v>
       </c>
@@ -652,7 +676,9 @@
       <c r="E11" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="F11" s="2"/>
+      <c r="F11" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H11" s="0" t="n">
         <v>0.2225</v>
       </c>
@@ -669,7 +695,7 @@
         <v>0.0356</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="n">
         <v>11</v>
       </c>
@@ -685,7 +711,9 @@
       <c r="E12" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="F12" s="2"/>
+      <c r="F12" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H12" s="0" t="n">
         <v>0.2182</v>
       </c>
@@ -702,7 +730,7 @@
         <v>0.0343</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="n">
         <v>12</v>
       </c>
@@ -718,7 +746,9 @@
       <c r="E13" s="0" t="n">
         <v>0</v>
       </c>
-      <c r="F13" s="2"/>
+      <c r="F13" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H13" s="0" t="n">
         <v>0.2989</v>
       </c>
@@ -735,7 +765,7 @@
         <v>0.0468</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="n">
         <v>13</v>
       </c>
@@ -751,7 +781,9 @@
       <c r="E14" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="F14" s="2"/>
+      <c r="F14" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H14" s="0" t="n">
         <v>0.2952</v>
       </c>
@@ -768,7 +800,7 @@
         <v>0.0457</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="n">
         <v>14</v>
       </c>
@@ -784,7 +816,9 @@
       <c r="E15" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="F15" s="2"/>
+      <c r="F15" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H15" s="0" t="n">
         <v>0.2914</v>
       </c>
@@ -801,7 +835,7 @@
         <v>0.0445</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="n">
         <v>15</v>
       </c>
@@ -817,7 +851,9 @@
       <c r="E16" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="F16" s="2"/>
+      <c r="F16" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H16" s="0" t="n">
         <v>0.2877</v>
       </c>
@@ -834,7 +870,7 @@
         <v>0.0434</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="n">
         <v>16</v>
       </c>
@@ -850,7 +886,9 @@
       <c r="E17" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="F17" s="2"/>
+      <c r="F17" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H17" s="0" t="n">
         <v>0.2839</v>
       </c>
@@ -867,7 +905,7 @@
         <v>0.0423</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="n">
         <v>17</v>
       </c>
@@ -883,7 +921,9 @@
       <c r="E18" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="F18" s="4"/>
+      <c r="F18" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="H18" s="0" t="n">
         <v>0.2801</v>
       </c>
@@ -900,7 +940,7 @@
         <v>0.0411</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="n">
         <v>18</v>
       </c>
@@ -916,7 +956,9 @@
       <c r="E19" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="F19" s="4"/>
+      <c r="F19" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="H19" s="0" t="n">
         <v>0.2764</v>
       </c>
@@ -933,7 +975,7 @@
         <v>0.04</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="n">
         <v>19</v>
       </c>
@@ -949,7 +991,9 @@
       <c r="E20" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="F20" s="2"/>
+      <c r="F20" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H20" s="0" t="n">
         <v>0.2726</v>
       </c>
@@ -966,7 +1010,7 @@
         <v>0.0389</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="n">
         <v>20</v>
       </c>
@@ -982,7 +1026,9 @@
       <c r="E21" s="0" t="n">
         <v>8</v>
       </c>
-      <c r="F21" s="2"/>
+      <c r="F21" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H21" s="0" t="n">
         <v>0.2689</v>
       </c>
@@ -999,7 +1045,7 @@
         <v>0.0377</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="n">
         <v>21</v>
       </c>
@@ -1015,7 +1061,9 @@
       <c r="E22" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="F22" s="2"/>
+      <c r="F22" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H22" s="0" t="n">
         <v>0.2651</v>
       </c>
@@ -1032,7 +1080,7 @@
         <v>0.0366</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="n">
         <v>22</v>
       </c>
@@ -1048,7 +1096,9 @@
       <c r="E23" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="F23" s="2"/>
+      <c r="F23" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H23" s="0" t="n">
         <v>0.2614</v>
       </c>
@@ -1065,7 +1115,7 @@
         <v>0.0355</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="n">
         <v>23</v>
       </c>
@@ -1081,7 +1131,9 @@
       <c r="E24" s="0" t="n">
         <v>0</v>
       </c>
-      <c r="F24" s="2"/>
+      <c r="F24" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H24" s="0" t="n">
         <v>0.3371</v>
       </c>
@@ -1098,7 +1150,7 @@
         <v>0.0464</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="n">
         <v>24</v>
       </c>
@@ -1114,7 +1166,9 @@
       <c r="E25" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="F25" s="2"/>
+      <c r="F25" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H25" s="0" t="n">
         <v>0.3338</v>
       </c>
@@ -1131,7 +1185,7 @@
         <v>0.0455</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="n">
         <v>25</v>
       </c>
@@ -1147,7 +1201,9 @@
       <c r="E26" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="F26" s="2"/>
+      <c r="F26" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H26" s="0" t="n">
         <v>0.3306</v>
       </c>
@@ -1164,7 +1220,7 @@
         <v>0.0445</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="n">
         <v>26</v>
       </c>
@@ -1180,7 +1236,9 @@
       <c r="E27" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="F27" s="2"/>
+      <c r="F27" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H27" s="0" t="n">
         <v>0.3273</v>
       </c>
@@ -1197,7 +1255,7 @@
         <v>0.0435</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="n">
         <v>27</v>
       </c>
@@ -1213,7 +1271,9 @@
       <c r="E28" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="F28" s="2"/>
+      <c r="F28" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H28" s="0" t="n">
         <v>0.324</v>
       </c>
@@ -1230,7 +1290,7 @@
         <v>0.0425</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="n">
         <v>28</v>
       </c>
@@ -1246,7 +1306,9 @@
       <c r="E29" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="F29" s="2"/>
+      <c r="F29" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H29" s="0" t="n">
         <v>0.3208</v>
       </c>
@@ -1263,7 +1325,7 @@
         <v>0.0415</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="n">
         <v>29</v>
       </c>
@@ -1279,7 +1341,9 @@
       <c r="E30" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="F30" s="2"/>
+      <c r="F30" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H30" s="0" t="n">
         <v>0.3175</v>
       </c>
@@ -1296,7 +1360,7 @@
         <v>0.0406</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="0" t="n">
         <v>30</v>
       </c>
@@ -1312,7 +1376,9 @@
       <c r="E31" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="F31" s="2"/>
+      <c r="F31" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H31" s="0" t="n">
         <v>0.3143</v>
       </c>
@@ -1329,7 +1395,7 @@
         <v>0.0396</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="0" t="n">
         <v>31</v>
       </c>
@@ -1345,7 +1411,9 @@
       <c r="E32" s="0" t="n">
         <v>8</v>
       </c>
-      <c r="F32" s="2"/>
+      <c r="F32" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H32" s="0" t="n">
         <v>0.311</v>
       </c>
@@ -1362,7 +1430,7 @@
         <v>0.0386</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="0" t="n">
         <v>32</v>
       </c>
@@ -1378,7 +1446,9 @@
       <c r="E33" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="F33" s="2"/>
+      <c r="F33" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H33" s="0" t="n">
         <v>0.3077</v>
       </c>
@@ -1395,7 +1465,7 @@
         <v>0.0376</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="n">
         <v>33</v>
       </c>
@@ -1411,7 +1481,9 @@
       <c r="E34" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="F34" s="2"/>
+      <c r="F34" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H34" s="0" t="n">
         <v>0.3045</v>
       </c>
@@ -1428,7 +1500,7 @@
         <v>0.0366</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="0" t="n">
         <v>34</v>
       </c>
@@ -1444,7 +1516,9 @@
       <c r="E35" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="F35" s="2"/>
+      <c r="F35" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H35" s="0" t="n">
         <v>0.3724</v>
       </c>
@@ -1461,7 +1535,7 @@
         <v>0.0453</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="0" t="n">
         <v>35</v>
       </c>
@@ -1477,7 +1551,9 @@
       <c r="E36" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="F36" s="2"/>
+      <c r="F36" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H36" s="0" t="n">
         <v>0.3697</v>
       </c>
@@ -1494,7 +1570,7 @@
         <v>0.0444</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="0" t="n">
         <v>36</v>
       </c>
@@ -1510,7 +1586,9 @@
       <c r="E37" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="F37" s="2"/>
+      <c r="F37" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H37" s="0" t="n">
         <v>0.3669</v>
       </c>
@@ -1527,7 +1605,7 @@
         <v>0.0436</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="0" t="n">
         <v>37</v>
       </c>
@@ -1543,7 +1621,9 @@
       <c r="E38" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="F38" s="2"/>
+      <c r="F38" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H38" s="0" t="n">
         <v>0.3642</v>
       </c>
@@ -1560,7 +1640,7 @@
         <v>0.0428</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="0" t="n">
         <v>38</v>
       </c>
@@ -1576,7 +1656,9 @@
       <c r="E39" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="F39" s="2"/>
+      <c r="F39" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H39" s="0" t="n">
         <v>0.3614</v>
       </c>
@@ -1593,7 +1675,7 @@
         <v>0.042</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="0" t="n">
         <v>39</v>
       </c>
@@ -1609,7 +1691,9 @@
       <c r="E40" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="F40" s="2"/>
+      <c r="F40" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H40" s="0" t="n">
         <v>0.3587</v>
       </c>
@@ -1626,7 +1710,7 @@
         <v>0.0411</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="0" t="n">
         <v>40</v>
       </c>
@@ -1642,7 +1726,9 @@
       <c r="E41" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="F41" s="2"/>
+      <c r="F41" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H41" s="0" t="n">
         <v>0.3559</v>
       </c>
@@ -1659,7 +1745,7 @@
         <v>0.0403</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="0" t="n">
         <v>41</v>
       </c>
@@ -1675,7 +1761,9 @@
       <c r="E42" s="0" t="n">
         <v>8</v>
       </c>
-      <c r="F42" s="2"/>
+      <c r="F42" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H42" s="0" t="n">
         <v>0.3531</v>
       </c>
@@ -1692,7 +1780,7 @@
         <v>0.0395</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="0" t="n">
         <v>42</v>
       </c>
@@ -1708,7 +1796,9 @@
       <c r="E43" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="F43" s="2"/>
+      <c r="F43" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H43" s="0" t="n">
         <v>0.3504</v>
       </c>
@@ -1725,7 +1815,7 @@
         <v>0.0387</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="0" t="n">
         <v>43</v>
       </c>
@@ -1741,7 +1831,9 @@
       <c r="E44" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="F44" s="2"/>
+      <c r="F44" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H44" s="0" t="n">
         <v>0.3476</v>
       </c>
@@ -1758,7 +1850,7 @@
         <v>0.0378</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="0" t="n">
         <v>44</v>
       </c>
@@ -1774,7 +1866,9 @@
       <c r="E45" s="0" t="n">
         <v>0</v>
       </c>
-      <c r="F45" s="2"/>
+      <c r="F45" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H45" s="0" t="n">
         <v>0.4133</v>
       </c>
@@ -1791,7 +1885,7 @@
         <v>0.0457</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="0" t="n">
         <v>45</v>
       </c>
@@ -1807,7 +1901,9 @@
       <c r="E46" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="F46" s="2"/>
+      <c r="F46" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H46" s="0" t="n">
         <v>0.4111</v>
       </c>
@@ -1824,7 +1920,7 @@
         <v>0.0451</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="0" t="n">
         <v>46</v>
       </c>
@@ -1840,7 +1936,9 @@
       <c r="E47" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="F47" s="2"/>
+      <c r="F47" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H47" s="0" t="n">
         <v>0.4088</v>
       </c>
@@ -1857,7 +1955,7 @@
         <v>0.0444</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="0" t="n">
         <v>47</v>
       </c>
@@ -1873,7 +1971,9 @@
       <c r="E48" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="F48" s="2"/>
+      <c r="F48" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H48" s="0" t="n">
         <v>0.4066</v>
       </c>
@@ -1890,7 +1990,7 @@
         <v>0.0437</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="0" t="n">
         <v>48</v>
       </c>
@@ -1906,7 +2006,9 @@
       <c r="E49" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="F49" s="2"/>
+      <c r="F49" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H49" s="0" t="n">
         <v>0.4043</v>
       </c>
@@ -1923,7 +2025,7 @@
         <v>0.0431</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="0" t="n">
         <v>49</v>
       </c>
@@ -1939,7 +2041,9 @@
       <c r="E50" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="F50" s="2"/>
+      <c r="F50" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H50" s="0" t="n">
         <v>0.402</v>
       </c>
@@ -1956,7 +2060,7 @@
         <v>0.0424</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="0" t="n">
         <v>50</v>
       </c>
@@ -1972,7 +2076,9 @@
       <c r="E51" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="F51" s="2"/>
+      <c r="F51" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H51" s="0" t="n">
         <v>0.3998</v>
       </c>
@@ -1989,7 +2095,7 @@
         <v>0.0417</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="0" t="n">
         <v>51</v>
       </c>
@@ -2005,7 +2111,9 @@
       <c r="E52" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="F52" s="2"/>
+      <c r="F52" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H52" s="0" t="n">
         <v>0.3975</v>
       </c>
@@ -2022,7 +2130,7 @@
         <v>0.041</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="0" t="n">
         <v>52</v>
       </c>
@@ -2038,7 +2146,9 @@
       <c r="E53" s="0" t="n">
         <v>0</v>
       </c>
-      <c r="F53" s="2"/>
+      <c r="F53" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H53" s="0" t="n">
         <v>0.4515</v>
       </c>
@@ -2055,7 +2165,7 @@
         <v>0.0454</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="0" t="n">
         <v>53</v>
       </c>
@@ -2071,7 +2181,9 @@
       <c r="E54" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="F54" s="2"/>
+      <c r="F54" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H54" s="0" t="n">
         <v>0.4497</v>
       </c>
@@ -2088,7 +2200,7 @@
         <v>0.0449</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="0" t="n">
         <v>54</v>
       </c>
@@ -2104,7 +2216,9 @@
       <c r="E55" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="F55" s="2"/>
+      <c r="F55" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H55" s="0" t="n">
         <v>0.448</v>
       </c>
@@ -2121,7 +2235,7 @@
         <v>0.0444</v>
       </c>
     </row>
-    <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="56" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="0" t="n">
         <v>55</v>
       </c>
@@ -2137,7 +2251,9 @@
       <c r="E56" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="F56" s="2"/>
+      <c r="F56" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H56" s="0" t="n">
         <v>0.4462</v>
       </c>
@@ -2154,7 +2270,7 @@
         <v>0.0438</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="0" t="n">
         <v>56</v>
       </c>
@@ -2170,7 +2286,9 @@
       <c r="E57" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="F57" s="2"/>
+      <c r="F57" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H57" s="0" t="n">
         <v>0.4444</v>
       </c>
@@ -2187,7 +2305,7 @@
         <v>0.0433</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="0" t="n">
         <v>57</v>
       </c>
@@ -2203,7 +2321,9 @@
       <c r="E58" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="F58" s="2"/>
+      <c r="F58" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H58" s="0" t="n">
         <v>0.4427</v>
       </c>
@@ -2220,7 +2340,7 @@
         <v>0.0428</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="0" t="n">
         <v>58</v>
       </c>
@@ -2236,7 +2356,9 @@
       <c r="E59" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="F59" s="2"/>
+      <c r="F59" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H59" s="0" t="n">
         <v>0.4409</v>
       </c>
@@ -2253,7 +2375,7 @@
         <v>0.0423</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="0" t="n">
         <v>59</v>
       </c>
@@ -2269,7 +2391,9 @@
       <c r="E60" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="F60" s="2"/>
+      <c r="F60" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H60" s="0" t="n">
         <v>0.4392</v>
       </c>
@@ -2286,7 +2410,7 @@
         <v>0.0418</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="0" t="n">
         <v>60</v>
       </c>
@@ -2302,7 +2426,9 @@
       <c r="E61" s="0" t="n">
         <v>0</v>
       </c>
-      <c r="F61" s="2"/>
+      <c r="F61" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H61" s="0" t="n">
         <v>0.4896</v>
       </c>
@@ -2319,7 +2445,7 @@
         <v>0.045</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="0" t="n">
         <v>61</v>
       </c>
@@ -2335,7 +2461,9 @@
       <c r="E62" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="F62" s="2"/>
+      <c r="F62" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H62" s="0" t="n">
         <v>0.4883</v>
       </c>
@@ -2352,7 +2480,7 @@
         <v>0.0447</v>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="63" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="0" t="n">
         <v>62</v>
       </c>
@@ -2368,7 +2496,9 @@
       <c r="E63" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="F63" s="2"/>
+      <c r="F63" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H63" s="0" t="n">
         <v>0.4871</v>
       </c>
@@ -2385,7 +2515,7 @@
         <v>0.0443</v>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="64" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="0" t="n">
         <v>63</v>
       </c>
@@ -2401,7 +2531,9 @@
       <c r="E64" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="F64" s="2"/>
+      <c r="F64" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H64" s="0" t="n">
         <v>0.4858</v>
       </c>
@@ -2418,7 +2550,7 @@
         <v>0.0439</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="65" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="0" t="n">
         <v>64</v>
       </c>
@@ -2434,7 +2566,9 @@
       <c r="E65" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="F65" s="2"/>
+      <c r="F65" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H65" s="0" t="n">
         <v>0.4846</v>
       </c>
@@ -2451,7 +2585,7 @@
         <v>0.0436</v>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="66" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="0" t="n">
         <v>65</v>
       </c>
@@ -2467,7 +2601,9 @@
       <c r="E66" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="F66" s="2"/>
+      <c r="F66" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H66" s="0" t="n">
         <v>0.4833</v>
       </c>
@@ -2484,7 +2620,7 @@
         <v>0.0432</v>
       </c>
     </row>
-    <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="67" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="0" t="n">
         <v>66</v>
       </c>
@@ -2500,7 +2636,9 @@
       <c r="E67" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="F67" s="2"/>
+      <c r="F67" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H67" s="0" t="n">
         <v>0.482</v>
       </c>
@@ -2517,7 +2655,7 @@
         <v>0.0429</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="68" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="0" t="n">
         <v>67</v>
       </c>
@@ -2533,7 +2671,9 @@
       <c r="E68" s="0" t="n">
         <v>0</v>
       </c>
-      <c r="F68" s="2"/>
+      <c r="F68" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H68" s="0" t="n">
         <v>0.5277</v>
       </c>
@@ -2550,7 +2690,7 @@
         <v>0.0447</v>
       </c>
     </row>
-    <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="69" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="0" t="n">
         <v>68</v>
       </c>
@@ -2566,7 +2706,9 @@
       <c r="E69" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="F69" s="2"/>
+      <c r="F69" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H69" s="0" t="n">
         <v>0.527</v>
       </c>
@@ -2583,7 +2725,7 @@
         <v>0.0445</v>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="70" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="0" t="n">
         <v>69</v>
       </c>
@@ -2599,7 +2741,9 @@
       <c r="E70" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="F70" s="2"/>
+      <c r="F70" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H70" s="0" t="n">
         <v>0.5262</v>
       </c>
@@ -2616,7 +2760,7 @@
         <v>0.0443</v>
       </c>
     </row>
-    <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="71" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="0" t="n">
         <v>70</v>
       </c>
@@ -2632,7 +2776,9 @@
       <c r="E71" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="F71" s="2"/>
+      <c r="F71" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H71" s="0" t="n">
         <v>0.5255</v>
       </c>
@@ -2649,7 +2795,7 @@
         <v>0.0441</v>
       </c>
     </row>
-    <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="72" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="0" t="n">
         <v>71</v>
       </c>
@@ -2665,7 +2811,9 @@
       <c r="E72" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="F72" s="2"/>
+      <c r="F72" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H72" s="0" t="n">
         <v>0.5247</v>
       </c>
@@ -2682,7 +2830,7 @@
         <v>0.0438</v>
       </c>
     </row>
-    <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="73" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="0" t="n">
         <v>72</v>
       </c>
@@ -2698,7 +2846,9 @@
       <c r="E73" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="F73" s="2"/>
+      <c r="F73" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H73" s="0" t="n">
         <v>0.5239</v>
       </c>
@@ -2715,7 +2865,7 @@
         <v>0.0436</v>
       </c>
     </row>
-    <row r="74" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="74" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="0" t="n">
         <v>73</v>
       </c>
@@ -2731,7 +2881,9 @@
       <c r="E74" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="F74" s="2"/>
+      <c r="F74" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H74" s="0" t="n">
         <v>0.5232</v>
       </c>
@@ -2748,7 +2900,7 @@
         <v>0.0434</v>
       </c>
     </row>
-    <row r="75" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="75" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="0" t="n">
         <v>74</v>
       </c>
@@ -2764,7 +2916,9 @@
       <c r="E75" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="F75" s="2"/>
+      <c r="F75" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H75" s="0" t="n">
         <v>0.5224</v>
       </c>
@@ -2781,7 +2935,7 @@
         <v>0.0432</v>
       </c>
     </row>
-    <row r="76" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="76" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="0" t="n">
         <v>75</v>
       </c>
@@ -2797,7 +2951,9 @@
       <c r="E76" s="0" t="n">
         <v>0</v>
       </c>
-      <c r="F76" s="2"/>
+      <c r="F76" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H76" s="0" t="n">
         <v>0.5659</v>
       </c>
@@ -2814,7 +2970,7 @@
         <v>0.0443</v>
       </c>
     </row>
-    <row r="77" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="77" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="0" t="n">
         <v>76</v>
       </c>
@@ -2830,7 +2986,9 @@
       <c r="E77" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="F77" s="2"/>
+      <c r="F77" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H77" s="0" t="n">
         <v>0.5656</v>
       </c>
@@ -2847,7 +3005,7 @@
         <v>0.0443</v>
       </c>
     </row>
-    <row r="78" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="78" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="0" t="n">
         <v>77</v>
       </c>
@@ -2863,7 +3021,9 @@
       <c r="E78" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="F78" s="2"/>
+      <c r="F78" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H78" s="0" t="n">
         <v>0.5653</v>
       </c>
@@ -2880,7 +3040,7 @@
         <v>0.0442</v>
       </c>
     </row>
-    <row r="79" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="79" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="0" t="n">
         <v>78</v>
       </c>
@@ -2896,7 +3056,9 @@
       <c r="E79" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="F79" s="2"/>
+      <c r="F79" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H79" s="0" t="n">
         <v>0.5651</v>
       </c>
@@ -2913,7 +3075,7 @@
         <v>0.0442</v>
       </c>
     </row>
-    <row r="80" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="80" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="0" t="n">
         <v>79</v>
       </c>
@@ -2929,7 +3091,9 @@
       <c r="E80" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="F80" s="2"/>
+      <c r="F80" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H80" s="0" t="n">
         <v>0.5648</v>
       </c>
@@ -2946,7 +3110,7 @@
         <v>0.0441</v>
       </c>
     </row>
-    <row r="81" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="81" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="0" t="n">
         <v>80</v>
       </c>
@@ -2962,7 +3126,9 @@
       <c r="E81" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="F81" s="2"/>
+      <c r="F81" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H81" s="0" t="n">
         <v>0.5646</v>
       </c>
@@ -2979,7 +3145,7 @@
         <v>0.0441</v>
       </c>
     </row>
-    <row r="82" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="82" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="0" t="n">
         <v>81</v>
       </c>
@@ -2995,7 +3161,9 @@
       <c r="E82" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="F82" s="2"/>
+      <c r="F82" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H82" s="0" t="n">
         <v>0.5643</v>
       </c>
@@ -3012,7 +3180,7 @@
         <v>0.044</v>
       </c>
     </row>
-    <row r="83" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="83" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="0" t="n">
         <v>82</v>
       </c>
@@ -3028,7 +3196,9 @@
       <c r="E83" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="F83" s="2"/>
+      <c r="F83" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H83" s="0" t="n">
         <v>0.5641</v>
       </c>
@@ -3045,7 +3215,7 @@
         <v>0.0439</v>
       </c>
     </row>
-    <row r="84" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="84" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="0" t="n">
         <v>83</v>
       </c>
@@ -3061,7 +3231,9 @@
       <c r="E84" s="0" t="n">
         <v>0</v>
       </c>
-      <c r="F84" s="2"/>
+      <c r="F84" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H84" s="0" t="n">
         <v>0.604</v>
       </c>
@@ -3078,7 +3250,7 @@
         <v>0.044</v>
       </c>
     </row>
-    <row r="85" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="85" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="0" t="n">
         <v>84</v>
       </c>
@@ -3094,7 +3266,9 @@
       <c r="E85" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="F85" s="2"/>
+      <c r="F85" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H85" s="0" t="n">
         <v>0.6042</v>
       </c>
@@ -3111,7 +3285,7 @@
         <v>0.0441</v>
       </c>
     </row>
-    <row r="86" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="86" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="0" t="n">
         <v>85</v>
       </c>
@@ -3127,7 +3301,9 @@
       <c r="E86" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="F86" s="2"/>
+      <c r="F86" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H86" s="0" t="n">
         <v>0.6045</v>
       </c>
@@ -3144,7 +3320,7 @@
         <v>0.0442</v>
       </c>
     </row>
-    <row r="87" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="87" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="0" t="n">
         <v>86</v>
       </c>
@@ -3160,7 +3336,9 @@
       <c r="E87" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="F87" s="2"/>
+      <c r="F87" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H87" s="0" t="n">
         <v>0.6047</v>
       </c>
@@ -3177,7 +3355,7 @@
         <v>0.0443</v>
       </c>
     </row>
-    <row r="88" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="88" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="0" t="n">
         <v>87</v>
       </c>
@@ -3193,7 +3371,9 @@
       <c r="E88" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="F88" s="2"/>
+      <c r="F88" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H88" s="0" t="n">
         <v>0.605</v>
       </c>
@@ -3210,7 +3390,7 @@
         <v>0.0444</v>
       </c>
     </row>
-    <row r="89" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="89" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="0" t="n">
         <v>88</v>
       </c>
@@ -3226,7 +3406,9 @@
       <c r="E89" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="F89" s="2"/>
+      <c r="F89" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H89" s="0" t="n">
         <v>0.6052</v>
       </c>
@@ -3243,7 +3425,7 @@
         <v>0.0445</v>
       </c>
     </row>
-    <row r="90" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="90" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="0" t="n">
         <v>89</v>
       </c>
@@ -3259,7 +3441,9 @@
       <c r="E90" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="F90" s="2"/>
+      <c r="F90" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H90" s="0" t="n">
         <v>0.6054</v>
       </c>
@@ -3276,7 +3460,7 @@
         <v>0.0446</v>
       </c>
     </row>
-    <row r="91" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="91" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="0" t="n">
         <v>90</v>
       </c>
@@ -3292,7 +3476,9 @@
       <c r="E91" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="F91" s="2"/>
+      <c r="F91" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H91" s="0" t="n">
         <v>0.6057</v>
       </c>
@@ -3309,7 +3495,7 @@
         <v>0.0447</v>
       </c>
     </row>
-    <row r="92" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="92" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="0" t="n">
         <v>91</v>
       </c>
@@ -3325,7 +3511,9 @@
       <c r="E92" s="0" t="n">
         <v>0</v>
       </c>
-      <c r="F92" s="2"/>
+      <c r="F92" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H92" s="0" t="n">
         <v>0.6421</v>
       </c>
@@ -3342,7 +3530,7 @@
         <v>0.0436</v>
       </c>
     </row>
-    <row r="93" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="93" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="0" t="n">
         <v>92</v>
       </c>
@@ -3358,7 +3546,9 @@
       <c r="E93" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="F93" s="2"/>
+      <c r="F93" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H93" s="0" t="n">
         <v>0.6429</v>
       </c>
@@ -3375,7 +3565,7 @@
         <v>0.0439</v>
       </c>
     </row>
-    <row r="94" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="94" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="0" t="n">
         <v>93</v>
       </c>
@@ -3391,7 +3581,9 @@
       <c r="E94" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="F94" s="2"/>
+      <c r="F94" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H94" s="0" t="n">
         <v>0.6436</v>
       </c>
@@ -3408,7 +3600,7 @@
         <v>0.0441</v>
       </c>
     </row>
-    <row r="95" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="95" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="0" t="n">
         <v>94</v>
       </c>
@@ -3424,7 +3616,9 @@
       <c r="E95" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="F95" s="2"/>
+      <c r="F95" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H95" s="0" t="n">
         <v>0.6444</v>
       </c>
@@ -3441,7 +3635,7 @@
         <v>0.0444</v>
       </c>
     </row>
-    <row r="96" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="96" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="0" t="n">
         <v>95</v>
       </c>
@@ -3457,7 +3651,9 @@
       <c r="E96" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="F96" s="2"/>
+      <c r="F96" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H96" s="0" t="n">
         <v>0.6451</v>
       </c>
@@ -3474,7 +3670,7 @@
         <v>0.0446</v>
       </c>
     </row>
-    <row r="97" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="97" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="0" t="n">
         <v>96</v>
       </c>
@@ -3490,7 +3686,9 @@
       <c r="E97" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="F97" s="2"/>
+      <c r="F97" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H97" s="0" t="n">
         <v>0.6458</v>
       </c>
@@ -3507,7 +3705,7 @@
         <v>0.0449</v>
       </c>
     </row>
-    <row r="98" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="98" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="0" t="n">
         <v>97</v>
       </c>
@@ -3523,7 +3721,9 @@
       <c r="E98" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="F98" s="2"/>
+      <c r="F98" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H98" s="0" t="n">
         <v>0.6466</v>
       </c>
@@ -3540,7 +3740,7 @@
         <v>0.0451</v>
       </c>
     </row>
-    <row r="99" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="99" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="0" t="n">
         <v>98</v>
       </c>
@@ -3556,7 +3756,9 @@
       <c r="E99" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="F99" s="2"/>
+      <c r="F99" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H99" s="0" t="n">
         <v>0.6473</v>
       </c>
@@ -3573,7 +3775,7 @@
         <v>0.0454</v>
       </c>
     </row>
-    <row r="100" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="100" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="0" t="n">
         <v>99</v>
       </c>
@@ -3589,7 +3791,9 @@
       <c r="E100" s="0" t="n">
         <v>8</v>
       </c>
-      <c r="F100" s="2"/>
+      <c r="F100" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H100" s="0" t="n">
         <v>0.6481</v>
       </c>
@@ -3606,7 +3810,7 @@
         <v>0.0456</v>
       </c>
     </row>
-    <row r="101" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="101" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="0" t="n">
         <v>100</v>
       </c>
@@ -3622,7 +3826,9 @@
       <c r="E101" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="F101" s="2"/>
+      <c r="F101" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H101" s="0" t="n">
         <v>0.6495</v>
       </c>

</xml_diff>

<commit_message>
Add basket recycle mode and working-cell replenishment
</commit_message>
<xml_diff>
--- a/fr3_real/fr3_100_cell_tracker.xlsx
+++ b/fr3_real/fr3_100_cell_tracker.xlsx
@@ -641,8 +641,8 @@
       <c r="E10" s="0" t="n">
         <v>8</v>
       </c>
-      <c r="F10" s="2" t="s">
-        <v>12</v>
+      <c r="F10" s="3" t="s">
+        <v>13</v>
       </c>
       <c r="H10" s="0" t="n">
         <v>0.2267</v>
@@ -676,8 +676,8 @@
       <c r="E11" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="F11" s="2" t="s">
-        <v>12</v>
+      <c r="F11" s="3" t="s">
+        <v>13</v>
       </c>
       <c r="H11" s="0" t="n">
         <v>0.2225</v>
@@ -3302,7 +3302,7 @@
         <v>2</v>
       </c>
       <c r="F86" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H86" s="0" t="n">
         <v>0.6045</v>

</xml_diff>